<commit_message>
Excel practice workbook: spread the decision dates across three statuses
Every deadline in the tracker had already lapsed relative to today, so
every row came out red and the exercise taught nothing. Dates now run
from June 2026 to January 2027, which yields lapsed, urgent and in-range
rows at once. Download links carry a version so nobody is served the old
file from cache.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/assets/Legal-Mind-family-workbook.xlsx
+++ b/excel/assets/Legal-Mind-family-workbook.xlsx
@@ -2141,7 +2141,6 @@
       </c>
       <c r="M29" s="2" t="n"/>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="C31" s="5" t="inlineStr">
         <is>
@@ -11133,7 +11132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -11190,7 +11189,7 @@
     </row>
     <row r="2">
       <c r="A2" s="11" t="n">
-        <v>45840</v>
+        <v>46175</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -11216,7 +11215,7 @@
     </row>
     <row r="3">
       <c r="A3" s="11" t="n">
-        <v>45853</v>
+        <v>46191</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -11242,7 +11241,7 @@
     </row>
     <row r="4">
       <c r="A4" s="11" t="n">
-        <v>45873</v>
+        <v>46209</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -11268,7 +11267,7 @@
     </row>
     <row r="5">
       <c r="A5" s="11" t="n">
-        <v>45895</v>
+        <v>46230</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
@@ -11294,7 +11293,7 @@
     </row>
     <row r="6">
       <c r="A6" s="11" t="n">
-        <v>45909</v>
+        <v>46236</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -11307,11 +11306,11 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>ימים קלנדריים</t>
+          <t>ימי עבודה</t>
         </is>
       </c>
       <c r="F6" s="11" t="n"/>
@@ -11320,7 +11319,7 @@
     </row>
     <row r="7">
       <c r="A7" s="11" t="n">
-        <v>45931</v>
+        <v>46240</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
@@ -11333,7 +11332,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -11346,7 +11345,7 @@
     </row>
     <row r="8">
       <c r="A8" s="11" t="n">
-        <v>45973</v>
+        <v>46258</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
@@ -11372,7 +11371,7 @@
     </row>
     <row r="9">
       <c r="A9" s="11" t="n">
-        <v>45994</v>
+        <v>46280</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -11385,11 +11384,11 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>ימי עבודה</t>
+          <t>ימים קלנדריים</t>
         </is>
       </c>
       <c r="F9" s="11" t="n"/>
@@ -11398,7 +11397,7 @@
     </row>
     <row r="10">
       <c r="A10" s="11" t="n">
-        <v>46036</v>
+        <v>46329</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -11424,7 +11423,7 @@
     </row>
     <row r="11">
       <c r="A11" s="11" t="n">
-        <v>46078</v>
+        <v>46399</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -11569,20 +11568,6 @@
     <row r="25">
       <c r="A25" s="15" t="n"/>
     </row>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Practice workbook: rebuild the expenses sheet, it was too obviously generated
Two artefacts of how I generated it: the payer was locked to the child, so
the mother paid only for one child and a pivot of payer by child came out
perfectly diagonal, and the amounts climbed by exactly 47 shekels a row.
Amounts now sit in plausible per-category ranges and the payer is
independent of the child. Every planted defect survives.

Adds a 59-check QA covering structure, formats, planted defects,
unintended artefacts such as arithmetic runs and perfect correlations,
cross-sheet consistency, plausibility, privacy and technical soundness.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/assets/Legal-Mind-family-workbook.xlsx
+++ b/excel/assets/Legal-Mind-family-workbook.xlsx
@@ -6755,16 +6755,16 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>הוצאות חינוך</t>
+          <t>חוגים</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>שכר לימוד</t>
+          <t>חוג כדורסל</t>
         </is>
       </c>
       <c r="E2" s="12" t="n">
-        <v>180</v>
+        <v>271</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -6773,12 +6773,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>לא</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>כן</t>
         </is>
       </c>
     </row>
@@ -6793,16 +6793,16 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>הוצאות רפואיות</t>
+          <t>ביגוד</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>משקפיים</t>
+          <t>ביגוד קיץ</t>
         </is>
       </c>
       <c r="E3" s="12" t="n">
-        <v>227</v>
+        <v>1070</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -6826,25 +6826,25 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>רומי</t>
+          <t>יהלי</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>חוגים</t>
+          <t>הוצאות חריגות</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>חוג ג'ודו</t>
+          <t>משקפי ראייה מיוחדים</t>
         </is>
       </c>
       <c r="E4" s="12" t="n">
-        <v>274</v>
+        <v>400</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -6864,21 +6864,21 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>נועה</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>ביגוד</t>
+          <t>הוצאות חינוך</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>ביגוד חורף</t>
+          <t>ספרי לימוד</t>
         </is>
       </c>
       <c r="E5" s="12" t="n">
-        <v>321</v>
+        <v>1094</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -6902,25 +6902,25 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>יהלי</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>נסיעות</t>
+          <t>חוגים</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>הסעה לבית ספר</t>
+          <t>חוג אמנות</t>
         </is>
       </c>
       <c r="E6" s="12" t="n">
-        <v>368</v>
+        <v>608</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -6945,16 +6945,16 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>מדור ואחזקת מדור</t>
+          <t>נסיעות</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>חשמל ומים</t>
+          <t>הסעה לבית ספר</t>
         </is>
       </c>
       <c r="E7" s="12" t="n">
-        <v>415</v>
+        <v>320</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -6963,7 +6963,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -6978,7 +6978,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>נועה</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -6988,20 +6988,20 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>מתנות לימי הולדת</t>
+          <t>אבחון דידקטי</t>
         </is>
       </c>
       <c r="E8" s="12" t="n">
-        <v>462</v>
+        <v>3600</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>האם</t>
+          <t>האב</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -7016,45 +7016,47 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>יהלי</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>הוצאות חינוך</t>
+          <t>הוצאות רפואיות</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>טיול שנתי</t>
+          <t>תרופות</t>
         </is>
       </c>
       <c r="E9" s="12" t="n">
-        <v>509</v>
+        <v>1010</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n">
-        <v>45439</v>
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>27.05.2024</t>
+        </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>רומי</t>
+          <t>נועה</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -7069,7 +7071,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>556</t>
+          <t>1680</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -7094,25 +7096,25 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>נועה</t>
+          <t>יהלי</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>חוגים</t>
+          <t>מדור ואחזקת מדור</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>חוג פסנתר</t>
+          <t>ארנונה</t>
         </is>
       </c>
       <c r="E11" s="12" t="n">
-        <v>603</v>
+        <v>1330</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>האם</t>
+          <t>האב</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -7132,7 +7134,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>יהלי</t>
+          <t>נועה</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -7142,15 +7144,15 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>נעליים</t>
+          <t>ציוד ספורט</t>
         </is>
       </c>
       <c r="E12" s="12" t="n">
-        <v>650</v>
+        <v>1070</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -7170,70 +7172,68 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>רומי</t>
+          <t>יהלי</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>נסיעות</t>
+          <t>הוצאות רפואיות</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>נסיעות לטיפולים</t>
+          <t>משקפיים</t>
         </is>
       </c>
       <c r="E13" s="12" t="n">
-        <v>697</v>
+        <v>1065</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
+          <t>האם</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="n">
+        <v>45467</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>נועה</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>מדור ואחזקת מדור</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>ועד בית</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>1390</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
           <t>האב</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>לא</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>24.06.2024</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>נועה</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>מדור ואחזקת מדור</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>חלק בשכר דירה</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="n">
-        <v>744</v>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>האם</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>כן</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -7248,21 +7248,21 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>יהלי</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>הוצאות חריגות</t>
+          <t>הוצאות חינוך</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>ציוד ספורט</t>
+          <t>ספרי לימוד</t>
         </is>
       </c>
       <c r="E15" s="12" t="n">
-        <v>791</v>
+        <v>865</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -7271,7 +7271,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -7291,30 +7291,30 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>הוצאות חינוך</t>
+          <t>חוגים</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>שיעור פרטי</t>
+          <t>חוג ג'ודו</t>
         </is>
       </c>
       <c r="E16" s="12" t="n">
-        <v>838</v>
+        <v>765</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
@@ -7324,7 +7324,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>נועה</t>
+          <t>יהלי</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -7334,11 +7334,11 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>טיפול שיניים</t>
+          <t>משקפיים</t>
         </is>
       </c>
       <c r="E17" s="12" t="n">
-        <v>885</v>
+        <v>225</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -7347,7 +7347,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -7362,30 +7362,30 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>יהלי</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>חוגים</t>
+          <t>מדור ואחזקת מדור</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>חוג כדורסל</t>
+          <t>ועד בית</t>
         </is>
       </c>
       <c r="E18" s="12" t="n">
-        <v>932</v>
+        <v>1755</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -7400,25 +7400,25 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>רומי</t>
+          <t>נועה</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>ביגוד</t>
+          <t>הוצאות רפואיות</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>ביגוד קיץ</t>
+          <t>רופא מומחה</t>
         </is>
       </c>
       <c r="E19" s="12" t="n">
-        <v>979</v>
+        <v>315</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -7438,25 +7438,25 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>נועה</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>נסיעות</t>
+          <t>הוצאות חינוך</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>הסעה לבית ספר</t>
+          <t>צהרון</t>
         </is>
       </c>
       <c r="E20" s="12" t="n">
-        <v>1026</v>
+        <v>1890</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>האם</t>
+          <t>האב</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -7466,7 +7466,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
@@ -7476,21 +7476,21 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>יהלי</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>מדור ואחזקת מדור</t>
+          <t>הוצאות חריגות</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>ארנונה</t>
+          <t>טיפול אורתודנטי</t>
         </is>
       </c>
       <c r="E21" s="12" t="n">
-        <v>1073</v>
+        <v>405</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -7514,30 +7514,30 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>רומי</t>
+          <t>נועה</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>הוצאות חריגות</t>
+          <t>הוצאות חינוך</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>מתנות לימי הולדת</t>
+          <t>טיול שנתי</t>
         </is>
       </c>
       <c r="E22" s="12" t="n">
-        <v>1120</v>
+        <v>1955</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -7552,7 +7552,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>נועה</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -7562,20 +7562,20 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>ספרי לימוד</t>
+          <t>טיול שנתי</t>
         </is>
       </c>
       <c r="E23" s="12" t="n">
-        <v>1167</v>
+        <v>3185</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>האם</t>
+          <t>האב</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -7590,35 +7590,35 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>יהלי</t>
+          <t>נועה</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>הוצאות רפואיות</t>
+          <t>הוצאות חינוך</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>פסיכולוג</t>
+          <t>ספרי לימוד</t>
         </is>
       </c>
       <c r="E24" s="12" t="n">
-        <v>1214</v>
+        <v>3290</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
           <t>לא</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>כן</t>
         </is>
       </c>
     </row>
@@ -7633,16 +7633,16 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>חוגים</t>
+          <t>הוצאות חריגות</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>מנוי בריכה</t>
+          <t>טיפול אורתודנטי</t>
         </is>
       </c>
       <c r="E25" s="12" t="n">
-        <v>1261</v>
+        <v>3255</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -7651,7 +7651,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -7671,20 +7671,20 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>ביגוד</t>
+          <t>הוצאות רפואיות</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>ביגוד חורף</t>
+          <t>רופא מומחה</t>
         </is>
       </c>
       <c r="E26" s="12" t="n">
-        <v>1308</v>
+        <v>715</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>האם</t>
+          <t>האב</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -7704,21 +7704,21 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>יהלי</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>נסיעות</t>
+          <t>הוצאות חינוך</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>נסיעות לטיפולים</t>
+          <t>שכר לימוד</t>
         </is>
       </c>
       <c r="E27" s="12" t="n">
-        <v>1355</v>
+        <v>990</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -7727,7 +7727,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -7742,21 +7742,21 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>רומי</t>
+          <t>יהלי</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>מדור ואחזקת מדור</t>
+          <t>חוגים</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>חשמל ומים</t>
+          <t>חוג ג'ודו</t>
         </is>
       </c>
       <c r="E28" s="12" t="n">
-        <v>1402</v>
+        <v>235</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -7785,20 +7785,20 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>הוצאות חריגות</t>
+          <t>הוצאות חינוך</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>ציוד ספורט</t>
+          <t>שיעור פרטי</t>
         </is>
       </c>
       <c r="E29" s="12" t="n">
-        <v>1449</v>
+        <v>1365</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>האם</t>
+          <t>האב</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -7808,7 +7808,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
@@ -7818,35 +7818,35 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>יהלי</t>
+          <t>נועה</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>הוצאות חינוך</t>
+          <t>ביגוד</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>צהרון</t>
+          <t>מעיל</t>
         </is>
       </c>
       <c r="E30" s="12" t="n">
-        <v>1496</v>
+        <v>990</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
@@ -7856,7 +7856,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>רומי</t>
+          <t>נועה</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -7866,11 +7866,11 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>קופת חולים</t>
+          <t>טיפול שיניים</t>
         </is>
       </c>
       <c r="E31" s="12" t="n">
-        <v>1543</v>
+        <v>1620</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -7894,25 +7894,25 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>נועה</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>חוגים</t>
+          <t>הוצאות חריגות</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>חוג ג'ודו</t>
+          <t>טיפול אורתודנטי</t>
         </is>
       </c>
       <c r="E32" s="12" t="n">
-        <v>190</v>
+        <v>2330</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>האם</t>
+          <t>האב</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -7922,7 +7922,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
@@ -7932,21 +7932,21 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>יהלי</t>
+          <t>נועה</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>ביגוד</t>
+          <t>הוצאות חריגות</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>נעליים</t>
+          <t>טיפול אורתודנטי</t>
         </is>
       </c>
       <c r="E33" s="12" t="n">
-        <v>237</v>
+        <v>2863</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -7960,7 +7960,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
@@ -7970,30 +7970,30 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>רומי</t>
+          <t>יהלי</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>נסיעות</t>
+          <t>הוצאות חינוך</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>הסעה לבית ספר</t>
+          <t>ספרי לימוד</t>
         </is>
       </c>
       <c r="E34" s="12" t="n">
-        <v>284</v>
+        <v>2775</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -8008,27 +8008,27 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>נועה</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>מדור ואחזקת מדור</t>
+          <t>חוגים</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>חלק בשכר דירה</t>
+          <t>מנוי בריכה</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>331</t>
+          <t>695</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>האם</t>
+          <t>האב</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -8038,7 +8038,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
@@ -8053,16 +8053,16 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>הוצאות חריגות</t>
+          <t>הוצאות רפואיות</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>מתנות לימי הולדת</t>
+          <t>טיפול שיניים</t>
         </is>
       </c>
       <c r="E36" s="12" t="n">
-        <v>378</v>
+        <v>312</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -8091,16 +8091,16 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>הוצאות חינוך</t>
+          <t>הוצאות חריגות</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>שכר לימוד</t>
+          <t>אבחון דידקטי</t>
         </is>
       </c>
       <c r="E37" s="12" t="n">
-        <v>425</v>
+        <v>1240</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -8109,12 +8109,12 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
           <t>לא</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>כן</t>
         </is>
       </c>
     </row>
@@ -8129,16 +8129,16 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>הוצאות רפואיות</t>
+          <t>נסיעות</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>משקפיים</t>
+          <t>הסעה לבית ספר</t>
         </is>
       </c>
       <c r="E38" s="12" t="n">
-        <v>472</v>
+        <v>195</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -8167,20 +8167,20 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>חוגים</t>
+          <t>מדור ואחזקת מדור</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>חוג פסנתר</t>
+          <t>חשמל ומים</t>
         </is>
       </c>
       <c r="E39" s="12" t="n">
-        <v>519</v>
+        <v>2040</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -8200,25 +8200,25 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>רומי</t>
+          <t>נועה</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>ביגוד</t>
+          <t>הוצאות חינוך</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>ביגוד קיץ</t>
+          <t>שכר לימוד</t>
         </is>
       </c>
       <c r="E40" s="12" t="n">
-        <v>566</v>
+        <v>495</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -8228,7 +8228,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
@@ -8238,21 +8238,21 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>נועה</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>נסיעות</t>
+          <t>ביגוד</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>נסיעות לטיפולים</t>
+          <t>ציוד ספורט</t>
         </is>
       </c>
       <c r="E41" s="12" t="n">
-        <v>613</v>
+        <v>795</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -8276,30 +8276,30 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>יהלי</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>מדור ואחזקת מדור</t>
+          <t>ביגוד</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>ארנונה</t>
+          <t>ביגוד חורף</t>
         </is>
       </c>
       <c r="E42" s="12" t="n">
-        <v>660</v>
+        <v>610</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -8321,20 +8321,20 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>הוצאות חריגות</t>
+          <t>חוגים</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>ציוד ספורט</t>
+          <t>מנוי בריכה</t>
         </is>
       </c>
       <c r="E43" s="12" t="n">
-        <v>707</v>
+        <v>792</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -8359,20 +8359,20 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>הוצאות חינוך</t>
+          <t>הוצאות חריגות</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>טיול שנתי</t>
+          <t>טיפול רגשי</t>
         </is>
       </c>
       <c r="E44" s="12" t="n">
-        <v>754</v>
+        <v>3541</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>האם</t>
+          <t>האב</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -8382,7 +8382,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
@@ -8392,21 +8392,21 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>יהלי</t>
+          <t>נועה</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>הוצאות רפואיות</t>
+          <t>ביגוד</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>תרופות</t>
+          <t>ביגוד חורף</t>
         </is>
       </c>
       <c r="E45" s="12" t="n">
-        <v>801</v>
+        <v>355</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -8420,7 +8420,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
@@ -8430,25 +8430,25 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>רומי</t>
+          <t>נועה</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>חוגים</t>
+          <t>מדור ואחזקת מדור</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>חוג כדורסל</t>
+          <t>ארנונה</t>
         </is>
       </c>
       <c r="E46" s="12" t="n">
-        <v>848</v>
+        <v>442</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -8468,30 +8468,30 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>נועה</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>ביגוד</t>
+          <t>נסיעות</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>ביגוד חורף</t>
+          <t>הסעה לבית ספר</t>
         </is>
       </c>
       <c r="E47" s="12" t="n">
-        <v>895</v>
+        <v>245</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>האם</t>
+          <t>האב</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -8511,20 +8511,20 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>נסיעות</t>
+          <t>הוצאות חריגות</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>הסעה לבית ספר</t>
+          <t>אבחון דידקטי</t>
         </is>
       </c>
       <c r="E48" s="12" t="n">
-        <v>942</v>
+        <v>3175</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -8544,21 +8544,21 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>רומי</t>
+          <t>נועה</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>מדור ואחזקת מדור</t>
+          <t>הוצאות רפואיות</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>חשמל ומים</t>
+          <t>פסיכולוג</t>
         </is>
       </c>
       <c r="E49" s="12" t="n">
-        <v>989</v>
+        <v>610</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -8582,30 +8582,30 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>נועה</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>הוצאות חריגות</t>
+          <t>ביגוד</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>מתנות לימי הולדת</t>
+          <t>מעיל</t>
         </is>
       </c>
       <c r="E50" s="12" t="n">
-        <v>1036</v>
+        <v>185</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>האם</t>
+          <t>האב</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -8625,16 +8625,16 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>הוצאות חינוך</t>
+          <t>ביגוד</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>שיעור פרטי</t>
+          <t>ביגוד קיץ</t>
         </is>
       </c>
       <c r="E51" s="12" t="n">
-        <v>1083</v>
+        <v>523</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -8643,12 +8643,12 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
@@ -8663,16 +8663,16 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>הוצאות רפואיות</t>
+          <t>מדור ואחזקת מדור</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>טיפול שיניים</t>
+          <t>ועד בית</t>
         </is>
       </c>
       <c r="E52" s="12" t="n">
-        <v>1130</v>
+        <v>1300</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -8681,7 +8681,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -8696,25 +8696,25 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>נועה</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>חוגים</t>
+          <t>הוצאות רפואיות</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>מנוי בריכה</t>
+          <t>טיפול שיניים</t>
         </is>
       </c>
       <c r="E53" s="12" t="n">
-        <v>1177</v>
+        <v>745</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>האם</t>
+          <t>האב</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -8734,7 +8734,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>יהלי</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -8744,15 +8744,15 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>נעליים</t>
+          <t>ביגוד חורף</t>
         </is>
       </c>
       <c r="E54" s="12" t="n">
-        <v>1224</v>
+        <v>770</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -8777,25 +8777,25 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>נסיעות</t>
+          <t>חוגים</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>נסיעות לטיפולים</t>
+          <t>חוג כדורסל</t>
         </is>
       </c>
       <c r="E55" s="12" t="n">
-        <v>1271</v>
+        <v>633</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -8810,25 +8810,25 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>נועה</t>
+          <t>יהלי</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>מדור ואחזקת מדור</t>
+          <t>הוצאות רפואיות</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>חלק בשכר דירה</t>
+          <t>טיפול שיניים</t>
         </is>
       </c>
       <c r="E56" s="12" t="n">
-        <v>1318</v>
+        <v>951</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>האם</t>
+          <t>האב</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -8848,25 +8848,25 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>יהלי</t>
+          <t>נועה</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>הוצאות חריגות</t>
+          <t>חוגים</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>ציוד ספורט</t>
+          <t>חוג כדורסל</t>
         </is>
       </c>
       <c r="E57" s="12" t="n">
-        <v>1365</v>
+        <v>430</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -8886,21 +8886,21 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>רומי</t>
+          <t>נועה</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>הוצאות חינוך</t>
+          <t>חוגים</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>ספרי לימוד</t>
+          <t>חוג אמנות</t>
         </is>
       </c>
       <c r="E58" s="12" t="n">
-        <v>1412</v>
+        <v>365</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -8909,12 +8909,12 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
@@ -8924,21 +8924,21 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>נועה</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>הוצאות רפואיות</t>
+          <t>ביגוד</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>פסיכולוג</t>
+          <t>ביגוד קיץ</t>
         </is>
       </c>
       <c r="E59" s="12" t="n">
-        <v>1459</v>
+        <v>720</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -8952,7 +8952,7 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
@@ -8962,21 +8962,21 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>יהלי</t>
+          <t>רומי</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>חוגים</t>
+          <t>מדור ואחזקת מדור</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>חוג ג'ודו</t>
+          <t>חלק בשכר דירה</t>
         </is>
       </c>
       <c r="E60" s="12" t="n">
-        <v>1506</v>
+        <v>1255</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -8985,7 +8985,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -9000,30 +9000,30 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>רומי</t>
+          <t>נועה</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>ביגוד</t>
+          <t>הוצאות רפואיות</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>ביגוד קיץ</t>
+          <t>פסיכולוג</t>
         </is>
       </c>
       <c r="E61" s="12" t="n">
-        <v>1553</v>
+        <v>1070</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -9038,25 +9038,25 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>רומי</t>
+          <t>נועה</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>ביגוד</t>
+          <t>הוצאות רפואיות</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>ביגוד קיץ</t>
+          <t>רופא מומחה</t>
         </is>
       </c>
       <c r="E62" s="12" t="n">
-        <v>979</v>
+        <v>315</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>האב</t>
+          <t>האם</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">

</xml_diff>